<commit_message>
Add flight test data for 2026-08-17/18/19, archive Pi backup files, restore pre/post-processing scripts
- Pull Landing telemetry, videos, and .ulg flight logs for 2026-08-17, 2026-08-18, 2026-08-19
- Move ~90 timestamped Pi backup (.bak_*) files into Hardware/scripts/archive/
- Restore scratchpad_validate_h_miscal.py and run_pxy_leakage_gtfb_ab.sh

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Hardware/docs/PLASMC_FoV_Gain_Sweep_2026-08-05.xlsx
+++ b/Hardware/docs/PLASMC_FoV_Gain_Sweep_2026-08-05.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="L:\Claude\Soft Landing\Hardware\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50B99489-3A48-44EF-8950-0024B25F0BD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6230A6A-AC74-479A-9085-A1A91B4001BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="141">
   <si>
     <t>Priority</t>
   </si>
@@ -463,7 +463,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -499,6 +499,13 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF9C4500"/>
+      <name val="Consolas"/>
+      <family val="3"/>
     </font>
   </fonts>
   <fills count="6">
@@ -560,7 +567,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -587,6 +594,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1141,13 +1151,13 @@
         <v>43</v>
       </c>
       <c r="F7" s="3"/>
-      <c r="G7" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="H7" s="3" t="s">
+      <c r="G7" s="9">
+        <v>0.7</v>
+      </c>
+      <c r="H7" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="I7" s="3" t="s">
+      <c r="I7" s="9" t="s">
         <v>17</v>
       </c>
       <c r="J7" s="3" t="s">
@@ -1170,20 +1180,20 @@
       <c r="C8" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="D8" s="10" t="s">
         <v>53</v>
       </c>
       <c r="E8" s="3" t="s">
         <v>54</v>
       </c>
       <c r="F8" s="3"/>
-      <c r="G8" s="3" t="s">
+      <c r="G8" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="H8" s="3" t="s">
+      <c r="H8" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="I8" s="3" t="s">
+      <c r="I8" s="9" t="s">
         <v>56</v>
       </c>
       <c r="J8" s="3" t="s">
@@ -1213,10 +1223,10 @@
         <v>54</v>
       </c>
       <c r="F9" s="3"/>
-      <c r="G9" s="3" t="s">
+      <c r="G9" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="H9" s="3" t="s">
+      <c r="H9" s="9" t="s">
         <v>18</v>
       </c>
       <c r="I9" s="3" t="s">

</xml_diff>